<commit_message>
feat(buqi): complete demo UI prefab set
</commit_message>
<xml_diff>
--- a/Design/Excel/GameHot/Datas/Game/UI.xlsx
+++ b/Design/Excel/GameHot/Datas/Game/UI.xlsx
@@ -1042,7 +1042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.872727272727269" defaultRowHeight="14"/>
   <cols>
     <col width="8.872727272727269" customWidth="1" style="3" min="1" max="1"/>
@@ -1523,6 +1523,130 @@
         <v>1</v>
       </c>
     </row>
+    <row r="15">
+      <c r="B15" s="3" t="n">
+        <v>104</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>BuqiRunShellForm</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>不器界面预览</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Hot/Buqi/BuqiRunShellForm</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="n">
+        <v>105</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>BuqiItemDetailForm</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>装备详情</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Hot/Buqi/BuqiItemDetailForm</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Pop</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H16" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="3" t="n">
+        <v>106</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>BuqiConfirmForm</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>不器确认框</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Hot/Buqi/BuqiConfirmForm</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Pop</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H17" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="3" t="n">
+        <v>107</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>BuqiMessageForm</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>不器状态提示</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Hot/Buqi/BuqiMessageForm</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>